<commit_message>
Change Postpaid Plan, Change Prepaid Pack, Add Add-On journeys; data-assumption audit fixes and guardrails
New Line Selection capability and the three Plans & Numbers journeys on shared steps. Audit: one definition each for service/line classification, an asset's plan, balance owed, ticket/order/SIM-swap/TON status, active service, business segment and fixed-line offers; Pre-to-Post picks the customer's own prepaid line; data engine honours the caller's id field; Appointment Booking, Drawer, Billing Account and capability samples; whole-dataset classification tests and source guards; data and business-rule guardrails in CLAUDE.md.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/Persona_Feature_Applicability_Matrix_Reference.xlsx
+++ b/vfq-dxp-app/reference/outputs/Persona_Feature_Applicability_Matrix_Reference.xlsx
@@ -17,8 +17,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roles &amp; Credentials'!$A$1:$S$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Applicability Matrix'!$A$2:$G$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Feature Inventory'!$A$1:$J$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Applicability Matrix'!$A$2:$G$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Feature Inventory'!$A$1:$J$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Legacy Crosswalk'!$A$1:$D$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -939,7 +939,7 @@
         </is>
       </c>
       <c r="P2" s="36" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="Q2" s="36" t="n">
         <v>64</v>
@@ -1030,7 +1030,7 @@
         </is>
       </c>
       <c r="P3" s="36" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="Q3" s="36" t="n">
         <v>41</v>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="P5" s="36" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="Q5" s="36" t="n">
         <v>31</v>
@@ -1303,7 +1303,7 @@
         </is>
       </c>
       <c r="P6" s="36" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="Q6" s="36" t="n">
         <v>54</v>
@@ -1940,7 +1940,7 @@
         </is>
       </c>
       <c r="P13" s="36" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="Q13" s="36" t="n">
         <v>18</v>
@@ -3312,7 +3312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG53"/>
+  <dimension ref="A1:AG56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.85" customWidth="1" min="1" max="1"/>
@@ -8397,8 +8397,241 @@
       <c r="AF53" s="56" t="n"/>
       <c r="AG53" s="56" t="n"/>
     </row>
+    <row r="54" ht="40.50" customHeight="1">
+      <c r="A54" s="53" t="inlineStr">
+        <is>
+          <t>FEAT-052</t>
+        </is>
+      </c>
+      <c r="B54" s="54" t="inlineStr">
+        <is>
+          <t>Mobile Postpaid</t>
+        </is>
+      </c>
+      <c r="C54" s="54" t="inlineStr">
+        <is>
+          <t>Change Postpaid Plan journey</t>
+        </is>
+      </c>
+      <c r="D54" s="54" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="E54" s="54" t="inlineStr">
+        <is>
+          <t>—  (routed directly)</t>
+        </is>
+      </c>
+      <c r="F54" s="54" t="inlineStr">
+        <is>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="G54" s="54" t="inlineStr"/>
+      <c r="H54" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I54" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J54" s="56" t="n"/>
+      <c r="K54" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L54" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M54" s="56" t="n"/>
+      <c r="N54" s="56" t="n"/>
+      <c r="O54" s="56" t="n"/>
+      <c r="P54" s="56" t="n"/>
+      <c r="Q54" s="56" t="n"/>
+      <c r="R54" s="56" t="n"/>
+      <c r="S54" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T54" s="56" t="n"/>
+      <c r="U54" s="56" t="n"/>
+      <c r="V54" s="56" t="n"/>
+      <c r="W54" s="56" t="n"/>
+      <c r="X54" s="56" t="n"/>
+      <c r="Y54" s="56" t="n"/>
+      <c r="Z54" s="56" t="n"/>
+      <c r="AA54" s="56" t="n"/>
+      <c r="AB54" s="56" t="n"/>
+      <c r="AC54" s="56" t="n"/>
+      <c r="AD54" s="56" t="n"/>
+      <c r="AE54" s="56" t="n"/>
+      <c r="AF54" s="56" t="n"/>
+      <c r="AG54" s="56" t="n"/>
+    </row>
+    <row r="55" ht="40.50" customHeight="1">
+      <c r="A55" s="53" t="inlineStr">
+        <is>
+          <t>FEAT-053</t>
+        </is>
+      </c>
+      <c r="B55" s="54" t="inlineStr">
+        <is>
+          <t>Mobile Prepaid</t>
+        </is>
+      </c>
+      <c r="C55" s="54" t="inlineStr">
+        <is>
+          <t>Change Prepaid Pack journey</t>
+        </is>
+      </c>
+      <c r="D55" s="54" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="E55" s="54" t="inlineStr">
+        <is>
+          <t>—  (routed directly)</t>
+        </is>
+      </c>
+      <c r="F55" s="54" t="inlineStr">
+        <is>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="G55" s="54" t="inlineStr"/>
+      <c r="H55" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I55" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J55" s="56" t="n"/>
+      <c r="K55" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L55" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M55" s="56" t="n"/>
+      <c r="N55" s="56" t="n"/>
+      <c r="O55" s="56" t="n"/>
+      <c r="P55" s="56" t="n"/>
+      <c r="Q55" s="56" t="n"/>
+      <c r="R55" s="56" t="n"/>
+      <c r="S55" s="56" t="n"/>
+      <c r="T55" s="56" t="n"/>
+      <c r="U55" s="56" t="n"/>
+      <c r="V55" s="56" t="n"/>
+      <c r="W55" s="56" t="n"/>
+      <c r="X55" s="56" t="n"/>
+      <c r="Y55" s="56" t="n"/>
+      <c r="Z55" s="56" t="n"/>
+      <c r="AA55" s="56" t="n"/>
+      <c r="AB55" s="56" t="n"/>
+      <c r="AC55" s="56" t="n"/>
+      <c r="AD55" s="56" t="n"/>
+      <c r="AE55" s="56" t="n"/>
+      <c r="AF55" s="56" t="n"/>
+      <c r="AG55" s="56" t="n"/>
+    </row>
+    <row r="56" ht="40.50" customHeight="1">
+      <c r="A56" s="53" t="inlineStr">
+        <is>
+          <t>FEAT-054</t>
+        </is>
+      </c>
+      <c r="B56" s="54" t="inlineStr">
+        <is>
+          <t>Mobile Postpaid</t>
+        </is>
+      </c>
+      <c r="C56" s="54" t="inlineStr">
+        <is>
+          <t>Add Add-On journey</t>
+        </is>
+      </c>
+      <c r="D56" s="54" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="E56" s="54" t="inlineStr">
+        <is>
+          <t>—  (routed directly)</t>
+        </is>
+      </c>
+      <c r="F56" s="54" t="inlineStr">
+        <is>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="G56" s="54" t="inlineStr"/>
+      <c r="H56" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I56" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J56" s="56" t="n"/>
+      <c r="K56" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L56" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M56" s="56" t="n"/>
+      <c r="N56" s="56" t="n"/>
+      <c r="O56" s="56" t="n"/>
+      <c r="P56" s="56" t="n"/>
+      <c r="Q56" s="56" t="n"/>
+      <c r="R56" s="56" t="n"/>
+      <c r="S56" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T56" s="56" t="n"/>
+      <c r="U56" s="56" t="n"/>
+      <c r="V56" s="56" t="n"/>
+      <c r="W56" s="56" t="n"/>
+      <c r="X56" s="56" t="n"/>
+      <c r="Y56" s="56" t="n"/>
+      <c r="Z56" s="56" t="n"/>
+      <c r="AA56" s="56" t="n"/>
+      <c r="AB56" s="56" t="n"/>
+      <c r="AC56" s="56" t="n"/>
+      <c r="AD56" s="56" t="n"/>
+      <c r="AE56" s="56" t="n"/>
+      <c r="AF56" s="56" t="n"/>
+      <c r="AG56" s="56" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:G53"/>
+  <autoFilter ref="A2:G56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9770,7 +10003,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.85" customWidth="1" min="1" max="1"/>
@@ -12207,8 +12440,146 @@
       </c>
       <c r="J52" s="39" t="inlineStr"/>
     </row>
+    <row r="53">
+      <c r="A53" s="39" t="inlineStr">
+        <is>
+          <t>FEAT-052</t>
+        </is>
+      </c>
+      <c r="B53" s="39" t="inlineStr">
+        <is>
+          <t>mobile.change-postpaid-plan</t>
+        </is>
+      </c>
+      <c r="C53" s="39" t="inlineStr">
+        <is>
+          <t>Change Postpaid Plan journey</t>
+        </is>
+      </c>
+      <c r="D53" s="39" t="inlineStr">
+        <is>
+          <t>Mobile Postpaid</t>
+        </is>
+      </c>
+      <c r="E53" s="36" t="inlineStr">
+        <is>
+          <t>workspace</t>
+        </is>
+      </c>
+      <c r="F53" s="36" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="G53" s="39" t="inlineStr">
+        <is>
+          <t>—  (routed directly)</t>
+        </is>
+      </c>
+      <c r="H53" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="I53" s="39" t="inlineStr">
+        <is>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="J53" s="39" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="39" t="inlineStr">
+        <is>
+          <t>FEAT-053</t>
+        </is>
+      </c>
+      <c r="B54" s="39" t="inlineStr">
+        <is>
+          <t>mobile.change-prepaid-pack</t>
+        </is>
+      </c>
+      <c r="C54" s="39" t="inlineStr">
+        <is>
+          <t>Change Prepaid Pack journey</t>
+        </is>
+      </c>
+      <c r="D54" s="39" t="inlineStr">
+        <is>
+          <t>Mobile Prepaid</t>
+        </is>
+      </c>
+      <c r="E54" s="36" t="inlineStr">
+        <is>
+          <t>workspace</t>
+        </is>
+      </c>
+      <c r="F54" s="36" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="G54" s="39" t="inlineStr">
+        <is>
+          <t>—  (routed directly)</t>
+        </is>
+      </c>
+      <c r="H54" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="I54" s="39" t="inlineStr">
+        <is>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="J54" s="39" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="39" t="inlineStr">
+        <is>
+          <t>FEAT-054</t>
+        </is>
+      </c>
+      <c r="B55" s="39" t="inlineStr">
+        <is>
+          <t>mobile.add-addon</t>
+        </is>
+      </c>
+      <c r="C55" s="39" t="inlineStr">
+        <is>
+          <t>Add Add-On journey</t>
+        </is>
+      </c>
+      <c r="D55" s="39" t="inlineStr">
+        <is>
+          <t>Mobile Postpaid</t>
+        </is>
+      </c>
+      <c r="E55" s="36" t="inlineStr">
+        <is>
+          <t>workspace</t>
+        </is>
+      </c>
+      <c r="F55" s="36" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="G55" s="39" t="inlineStr">
+        <is>
+          <t>—  (routed directly)</t>
+        </is>
+      </c>
+      <c r="H55" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="I55" s="39" t="inlineStr">
+        <is>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="J55" s="39" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J52"/>
+  <autoFilter ref="A1:J55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16392,7 +16763,7 @@
       </c>
       <c r="B31" s="70" t="inlineStr">
         <is>
-          <t>51 catalogued (38 built, 13 planned).</t>
+          <t>54 catalogued (41 built, 13 planned).</t>
         </is>
       </c>
     </row>
@@ -16492,7 +16863,7 @@
       </c>
       <c r="B41" t="inlineStr" s="44">
         <is>
-          <t>d47045d</t>
+          <t>50e8577</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actions drawer/menu: per-action icon tiles; drop Gold Number from line actions, FNP to fibre, merge SIM Replacement/Swap; untrack unused reference screenshots/deliverables
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/Persona_Feature_Applicability_Matrix_Reference.xlsx
+++ b/vfq-dxp-app/reference/outputs/Persona_Feature_Applicability_Matrix_Reference.xlsx
@@ -15640,7 +15640,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="T20" s="56" t="n"/>
+      <c r="T20" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="U20" s="55" t="inlineStr">
         <is>
           <t>✓</t>
@@ -16863,7 +16867,7 @@
       </c>
       <c r="B41" t="inlineStr" s="44">
         <is>
-          <t>beacb97</t>
+          <t>97435c0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Credit-limit rules (defaults, options, locks, breakdown, HRN fee exemption, Big Data credit risk, audit trail) held consistently across journeys and screens; protected-segment access; QID/Passport reconciliation; ID reconciliation vs MOI; Credit Control ID-type approval; ID expiry rule
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/Persona_Feature_Applicability_Matrix_Reference.xlsx
+++ b/vfq-dxp-app/reference/outputs/Persona_Feature_Applicability_Matrix_Reference.xlsx
@@ -1947,7 +1947,7 @@
       </c>
       <c r="R13" s="39" t="inlineStr">
         <is>
-          <t>agent-self-service, edit-customer-records, view-bell-notifications, ticket-audit-trail</t>
+          <t>agent-self-service, edit-customer-records, view-bell-notifications, ticket-audit-trail, view-safwa-customers, view-safwa-plus-customers, view-royal-customers</t>
         </is>
       </c>
       <c r="S13" s="39" t="inlineStr">
@@ -8642,7 +8642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.15" customWidth="1" min="1" max="1"/>
@@ -8659,6 +8659,9 @@
     <col width="22.95" customWidth="1" min="12" max="12"/>
     <col width="22.95" customWidth="1" min="13" max="13"/>
     <col width="22.95" customWidth="1" min="14" max="14"/>
+    <col width="22.95" customWidth="1" min="15" max="15"/>
+    <col width="22.95" customWidth="1" min="16" max="16"/>
+    <col width="22.95" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="86.40" customHeight="1">
@@ -8730,6 +8733,21 @@
       <c r="N1" s="58" t="inlineStr">
         <is>
           <t>view-bell-notifications</t>
+        </is>
+      </c>
+      <c r="O1" s="58" t="inlineStr">
+        <is>
+          <t>view-royal-customers</t>
+        </is>
+      </c>
+      <c r="P1" s="58" t="inlineStr">
+        <is>
+          <t>view-safwa-customers</t>
+        </is>
+      </c>
+      <c r="Q1" s="58" t="inlineStr">
+        <is>
+          <t>view-safwa-plus-customers</t>
         </is>
       </c>
     </row>
@@ -8776,6 +8794,9 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="O2" s="56" t="n"/>
+      <c r="P2" s="56" t="n"/>
+      <c r="Q2" s="56" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="59" t="inlineStr">
@@ -8820,6 +8841,9 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="O3" s="56" t="n"/>
+      <c r="P3" s="56" t="n"/>
+      <c r="Q3" s="56" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="59" t="inlineStr">
@@ -8864,6 +8888,9 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="O4" s="56" t="n"/>
+      <c r="P4" s="56" t="n"/>
+      <c r="Q4" s="56" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="59" t="inlineStr">
@@ -8904,6 +8931,9 @@
       <c r="L5" s="56" t="n"/>
       <c r="M5" s="56" t="n"/>
       <c r="N5" s="56" t="n"/>
+      <c r="O5" s="56" t="n"/>
+      <c r="P5" s="56" t="n"/>
+      <c r="Q5" s="56" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="59" t="inlineStr">
@@ -8948,6 +8978,9 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="O6" s="56" t="n"/>
+      <c r="P6" s="56" t="n"/>
+      <c r="Q6" s="56" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="59" t="inlineStr">
@@ -8992,6 +9025,9 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="O7" s="56" t="n"/>
+      <c r="P7" s="56" t="n"/>
+      <c r="Q7" s="56" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="59" t="inlineStr">
@@ -9036,6 +9072,9 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="O8" s="56" t="n"/>
+      <c r="P8" s="56" t="n"/>
+      <c r="Q8" s="56" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="59" t="inlineStr">
@@ -9076,6 +9115,9 @@
       <c r="L9" s="56" t="n"/>
       <c r="M9" s="56" t="n"/>
       <c r="N9" s="56" t="n"/>
+      <c r="O9" s="56" t="n"/>
+      <c r="P9" s="56" t="n"/>
+      <c r="Q9" s="56" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="59" t="inlineStr">
@@ -9108,6 +9150,9 @@
       <c r="L10" s="56" t="n"/>
       <c r="M10" s="56" t="n"/>
       <c r="N10" s="56" t="n"/>
+      <c r="O10" s="56" t="n"/>
+      <c r="P10" s="56" t="n"/>
+      <c r="Q10" s="56" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="59" t="inlineStr">
@@ -9156,6 +9201,9 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="O11" s="56" t="n"/>
+      <c r="P11" s="56" t="n"/>
+      <c r="Q11" s="56" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="59" t="inlineStr">
@@ -9204,6 +9252,9 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="O12" s="56" t="n"/>
+      <c r="P12" s="56" t="n"/>
+      <c r="Q12" s="56" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="59" t="inlineStr">
@@ -9252,6 +9303,21 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="O13" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P13" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Q13" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="59" t="inlineStr">
@@ -9300,6 +9366,9 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="O14" s="56" t="n"/>
+      <c r="P14" s="56" t="n"/>
+      <c r="Q14" s="56" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="59" t="inlineStr">
@@ -9344,6 +9413,9 @@
       <c r="L15" s="56" t="n"/>
       <c r="M15" s="56" t="n"/>
       <c r="N15" s="56" t="n"/>
+      <c r="O15" s="56" t="n"/>
+      <c r="P15" s="56" t="n"/>
+      <c r="Q15" s="56" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="59" t="inlineStr">
@@ -9388,6 +9460,9 @@
       <c r="L16" s="56" t="n"/>
       <c r="M16" s="56" t="n"/>
       <c r="N16" s="56" t="n"/>
+      <c r="O16" s="56" t="n"/>
+      <c r="P16" s="56" t="n"/>
+      <c r="Q16" s="56" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="59" t="inlineStr">
@@ -9432,6 +9507,9 @@
       <c r="L17" s="56" t="n"/>
       <c r="M17" s="56" t="n"/>
       <c r="N17" s="56" t="n"/>
+      <c r="O17" s="56" t="n"/>
+      <c r="P17" s="56" t="n"/>
+      <c r="Q17" s="56" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="59" t="inlineStr">
@@ -9476,6 +9554,9 @@
       <c r="L18" s="56" t="n"/>
       <c r="M18" s="56" t="n"/>
       <c r="N18" s="56" t="n"/>
+      <c r="O18" s="56" t="n"/>
+      <c r="P18" s="56" t="n"/>
+      <c r="Q18" s="56" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="59" t="inlineStr">
@@ -9524,6 +9605,9 @@
       <c r="L19" s="56" t="n"/>
       <c r="M19" s="56" t="n"/>
       <c r="N19" s="56" t="n"/>
+      <c r="O19" s="56" t="n"/>
+      <c r="P19" s="56" t="n"/>
+      <c r="Q19" s="56" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="59" t="inlineStr">
@@ -9572,6 +9656,9 @@
       <c r="L20" s="56" t="n"/>
       <c r="M20" s="56" t="n"/>
       <c r="N20" s="56" t="n"/>
+      <c r="O20" s="56" t="n"/>
+      <c r="P20" s="56" t="n"/>
+      <c r="Q20" s="56" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="59" t="inlineStr">
@@ -9624,6 +9711,9 @@
       </c>
       <c r="M21" s="56" t="n"/>
       <c r="N21" s="56" t="n"/>
+      <c r="O21" s="56" t="n"/>
+      <c r="P21" s="56" t="n"/>
+      <c r="Q21" s="56" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="59" t="inlineStr">
@@ -9660,6 +9750,9 @@
       <c r="L22" s="56" t="n"/>
       <c r="M22" s="56" t="n"/>
       <c r="N22" s="56" t="n"/>
+      <c r="O22" s="56" t="n"/>
+      <c r="P22" s="56" t="n"/>
+      <c r="Q22" s="56" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="59" t="inlineStr">
@@ -9732,6 +9825,9 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="O23" s="56" t="n"/>
+      <c r="P23" s="56" t="n"/>
+      <c r="Q23" s="56" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="59" t="inlineStr">
@@ -9804,6 +9900,9 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="O24" s="56" t="n"/>
+      <c r="P24" s="56" t="n"/>
+      <c r="Q24" s="56" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="59" t="inlineStr">
@@ -9848,6 +9947,9 @@
       <c r="L25" s="56" t="n"/>
       <c r="M25" s="56" t="n"/>
       <c r="N25" s="56" t="n"/>
+      <c r="O25" s="56" t="n"/>
+      <c r="P25" s="56" t="n"/>
+      <c r="Q25" s="56" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="59" t="inlineStr">
@@ -9884,6 +9986,9 @@
       <c r="L26" s="56" t="n"/>
       <c r="M26" s="56" t="n"/>
       <c r="N26" s="56" t="n"/>
+      <c r="O26" s="56" t="n"/>
+      <c r="P26" s="56" t="n"/>
+      <c r="Q26" s="56" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="59" t="inlineStr">
@@ -9936,6 +10041,9 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="O27" s="56" t="n"/>
+      <c r="P27" s="56" t="n"/>
+      <c r="Q27" s="56" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="44"/>
@@ -9952,6 +10060,9 @@
       <c r="L28" s="44"/>
       <c r="M28" s="44"/>
       <c r="N28" s="44"/>
+      <c r="O28" s="44"/>
+      <c r="P28" s="44"/>
+      <c r="Q28" s="44"/>
     </row>
     <row r="29">
       <c r="A29" s="45" t="inlineStr">
@@ -9972,6 +10083,9 @@
       <c r="L29" s="44"/>
       <c r="M29" s="44"/>
       <c r="N29" s="44"/>
+      <c r="O29" s="44"/>
+      <c r="P29" s="44"/>
+      <c r="Q29" s="44"/>
     </row>
     <row r="30">
       <c r="A30" s="44"/>
@@ -9988,6 +10102,9 @@
       <c r="L30" s="44"/>
       <c r="M30" s="44"/>
       <c r="N30" s="44"/>
+      <c r="O30" s="44"/>
+      <c r="P30" s="44"/>
+      <c r="Q30" s="44"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -16867,7 +16984,7 @@
       </c>
       <c r="B41" t="inlineStr" s="44">
         <is>
-          <t>97435c0</t>
+          <t>f519568</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bill Formatter page addition
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/Persona_Feature_Applicability_Matrix_Reference.xlsx
+++ b/vfq-dxp-app/reference/outputs/Persona_Feature_Applicability_Matrix_Reference.xlsx
@@ -14202,7 +14202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W33"/>
+  <dimension ref="A1:X33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.15" customWidth="1" min="1" max="1"/>
@@ -14228,6 +14228,7 @@
     <col width="7.43" customWidth="1" min="21" max="21"/>
     <col width="7.43" customWidth="1" min="22" max="22"/>
     <col width="7.43" customWidth="1" min="23" max="23"/>
+    <col width="7.43" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="202.50" customHeight="1">
@@ -14303,45 +14304,50 @@
       </c>
       <c r="O1" s="58" t="inlineStr">
         <is>
+          <t>Bill Formatter</t>
+        </is>
+      </c>
+      <c r="P1" s="58" t="inlineStr">
+        <is>
           <t>Administration</t>
         </is>
       </c>
-      <c r="P1" s="58" t="inlineStr">
+      <c r="Q1" s="58" t="inlineStr">
         <is>
           <t>Plans &amp; Numbers</t>
         </is>
       </c>
-      <c r="Q1" s="58" t="inlineStr">
+      <c r="R1" s="58" t="inlineStr">
         <is>
           <t>Service Management</t>
         </is>
       </c>
-      <c r="R1" s="58" t="inlineStr">
+      <c r="S1" s="58" t="inlineStr">
         <is>
           <t>Customer &amp; Account</t>
         </is>
       </c>
-      <c r="S1" s="58" t="inlineStr">
+      <c r="T1" s="58" t="inlineStr">
         <is>
           <t>Support &amp; Requests</t>
         </is>
       </c>
-      <c r="T1" s="58" t="inlineStr">
+      <c r="U1" s="58" t="inlineStr">
         <is>
           <t>Plans &amp; Installation</t>
         </is>
       </c>
-      <c r="U1" s="58" t="inlineStr">
+      <c r="V1" s="58" t="inlineStr">
         <is>
           <t>Service Management</t>
         </is>
       </c>
-      <c r="V1" s="58" t="inlineStr">
+      <c r="W1" s="58" t="inlineStr">
         <is>
           <t>Customer &amp; Account</t>
         </is>
       </c>
-      <c r="W1" s="58" t="inlineStr">
+      <c r="X1" s="58" t="inlineStr">
         <is>
           <t>Support &amp; Requests</t>
         </is>
@@ -14404,45 +14410,50 @@
       </c>
       <c r="O2" s="61" t="inlineStr">
         <is>
+          <t>bill-formatter</t>
+        </is>
+      </c>
+      <c r="P2" s="61" t="inlineStr">
+        <is>
           <t>administration</t>
         </is>
       </c>
-      <c r="P2" s="61" t="inlineStr">
+      <c r="Q2" s="61" t="inlineStr">
         <is>
           <t>mobile.plans-numbers</t>
         </is>
       </c>
-      <c r="Q2" s="61" t="inlineStr">
+      <c r="R2" s="61" t="inlineStr">
         <is>
           <t>mobile.service-management</t>
         </is>
       </c>
-      <c r="R2" s="61" t="inlineStr">
+      <c r="S2" s="61" t="inlineStr">
         <is>
           <t>mobile.customer-account</t>
         </is>
       </c>
-      <c r="S2" s="61" t="inlineStr">
+      <c r="T2" s="61" t="inlineStr">
         <is>
           <t>mobile.support-requests</t>
         </is>
       </c>
-      <c r="T2" s="61" t="inlineStr">
+      <c r="U2" s="61" t="inlineStr">
         <is>
           <t>fibre-home.plans-installation</t>
         </is>
       </c>
-      <c r="U2" s="61" t="inlineStr">
+      <c r="V2" s="61" t="inlineStr">
         <is>
           <t>fibre-home.service-management</t>
         </is>
       </c>
-      <c r="V2" s="61" t="inlineStr">
+      <c r="W2" s="61" t="inlineStr">
         <is>
           <t>fibre-home.customer-account</t>
         </is>
       </c>
-      <c r="W2" s="61" t="inlineStr">
+      <c r="X2" s="61" t="inlineStr">
         <is>
           <t>fibre-home.support-requests</t>
         </is>
@@ -14509,45 +14520,50 @@
       </c>
       <c r="O3" s="64" t="inlineStr">
         <is>
+          <t>approach ordering (IA only)</t>
+        </is>
+      </c>
+      <c r="P3" s="64" t="inlineStr">
+        <is>
           <t>feature grant: workspace.admin-role-access-viewer</t>
         </is>
       </c>
-      <c r="P3" s="64" t="inlineStr">
+      <c r="Q3" s="64" t="inlineStr">
         <is>
           <t>journey grants in this category</t>
         </is>
       </c>
-      <c r="Q3" s="64" t="inlineStr">
+      <c r="R3" s="64" t="inlineStr">
         <is>
           <t>journey grants in this category</t>
         </is>
       </c>
-      <c r="R3" s="64" t="inlineStr">
+      <c r="S3" s="64" t="inlineStr">
         <is>
           <t>journey grants in this category</t>
         </is>
       </c>
-      <c r="S3" s="64" t="inlineStr">
+      <c r="T3" s="64" t="inlineStr">
         <is>
           <t>journey grants in this category</t>
         </is>
       </c>
-      <c r="T3" s="64" t="inlineStr">
+      <c r="U3" s="64" t="inlineStr">
         <is>
           <t>journey grants in this category</t>
         </is>
       </c>
-      <c r="U3" s="64" t="inlineStr">
+      <c r="V3" s="64" t="inlineStr">
         <is>
           <t>journey grants in this category</t>
         </is>
       </c>
-      <c r="V3" s="64" t="inlineStr">
+      <c r="W3" s="64" t="inlineStr">
         <is>
           <t>journey grants in this category</t>
         </is>
       </c>
-      <c r="W3" s="64" t="inlineStr">
+      <c r="X3" s="64" t="inlineStr">
         <is>
           <t>journey grants in this category</t>
         </is>
@@ -14624,12 +14640,12 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O4" s="56" t="n"/>
-      <c r="P4" s="55" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="O4" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P4" s="56" t="n"/>
       <c r="Q4" s="55" t="inlineStr">
         <is>
           <t>✓</t>
@@ -14661,6 +14677,11 @@
         </is>
       </c>
       <c r="W4" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X4" s="55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -14717,7 +14738,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O5" s="56" t="n"/>
+      <c r="O5" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P5" s="56" t="n"/>
       <c r="Q5" s="56" t="n"/>
       <c r="R5" s="56" t="n"/>
@@ -14726,6 +14751,7 @@
       <c r="U5" s="56" t="n"/>
       <c r="V5" s="56" t="n"/>
       <c r="W5" s="56" t="n"/>
+      <c r="X5" s="56" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="59" t="inlineStr">
@@ -14778,7 +14804,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O6" s="56" t="n"/>
+      <c r="O6" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P6" s="56" t="n"/>
       <c r="Q6" s="56" t="n"/>
       <c r="R6" s="56" t="n"/>
@@ -14787,6 +14817,7 @@
       <c r="U6" s="56" t="n"/>
       <c r="V6" s="56" t="n"/>
       <c r="W6" s="56" t="n"/>
+      <c r="X6" s="56" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="59" t="inlineStr">
@@ -14839,7 +14870,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O7" s="56" t="n"/>
+      <c r="O7" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P7" s="56" t="n"/>
       <c r="Q7" s="56" t="n"/>
       <c r="R7" s="56" t="n"/>
@@ -14848,6 +14883,7 @@
       <c r="U7" s="56" t="n"/>
       <c r="V7" s="56" t="n"/>
       <c r="W7" s="56" t="n"/>
+      <c r="X7" s="56" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="59" t="inlineStr">
@@ -14900,7 +14936,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O8" s="56" t="n"/>
+      <c r="O8" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P8" s="56" t="n"/>
       <c r="Q8" s="56" t="n"/>
       <c r="R8" s="56" t="n"/>
@@ -14909,6 +14949,7 @@
       <c r="U8" s="56" t="n"/>
       <c r="V8" s="56" t="n"/>
       <c r="W8" s="56" t="n"/>
+      <c r="X8" s="56" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="59" t="inlineStr">
@@ -14961,7 +15002,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O9" s="56" t="n"/>
+      <c r="O9" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P9" s="56" t="n"/>
       <c r="Q9" s="56" t="n"/>
       <c r="R9" s="56" t="n"/>
@@ -14970,6 +15015,7 @@
       <c r="U9" s="56" t="n"/>
       <c r="V9" s="56" t="n"/>
       <c r="W9" s="56" t="n"/>
+      <c r="X9" s="56" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="59" t="inlineStr">
@@ -15022,7 +15068,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O10" s="56" t="n"/>
+      <c r="O10" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P10" s="56" t="n"/>
       <c r="Q10" s="56" t="n"/>
       <c r="R10" s="56" t="n"/>
@@ -15031,6 +15081,7 @@
       <c r="U10" s="56" t="n"/>
       <c r="V10" s="56" t="n"/>
       <c r="W10" s="56" t="n"/>
+      <c r="X10" s="56" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="59" t="inlineStr">
@@ -15103,31 +15154,36 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O11" s="56" t="n"/>
+      <c r="O11" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P11" s="56" t="n"/>
-      <c r="Q11" s="55" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="Q11" s="56" t="n"/>
       <c r="R11" s="55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="S11" s="56" t="n"/>
+      <c r="S11" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="T11" s="56" t="n"/>
-      <c r="U11" s="55" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="U11" s="56" t="n"/>
       <c r="V11" s="55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="W11" s="56" t="n"/>
+      <c r="W11" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X11" s="56" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="59" t="inlineStr">
@@ -15180,7 +15236,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O12" s="56" t="n"/>
+      <c r="O12" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P12" s="56" t="n"/>
       <c r="Q12" s="56" t="n"/>
       <c r="R12" s="56" t="n"/>
@@ -15189,6 +15249,7 @@
       <c r="U12" s="56" t="n"/>
       <c r="V12" s="56" t="n"/>
       <c r="W12" s="56" t="n"/>
+      <c r="X12" s="56" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="59" t="inlineStr">
@@ -15241,7 +15302,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O13" s="56" t="n"/>
+      <c r="O13" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P13" s="56" t="n"/>
       <c r="Q13" s="56" t="n"/>
       <c r="R13" s="56" t="n"/>
@@ -15250,6 +15315,7 @@
       <c r="U13" s="56" t="n"/>
       <c r="V13" s="56" t="n"/>
       <c r="W13" s="56" t="n"/>
+      <c r="X13" s="56" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="59" t="inlineStr">
@@ -15302,7 +15368,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O14" s="56" t="n"/>
+      <c r="O14" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P14" s="56" t="n"/>
       <c r="Q14" s="56" t="n"/>
       <c r="R14" s="56" t="n"/>
@@ -15311,6 +15381,7 @@
       <c r="U14" s="56" t="n"/>
       <c r="V14" s="56" t="n"/>
       <c r="W14" s="56" t="n"/>
+      <c r="X14" s="56" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="59" t="inlineStr">
@@ -15363,7 +15434,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O15" s="56" t="n"/>
+      <c r="O15" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P15" s="56" t="n"/>
       <c r="Q15" s="56" t="n"/>
       <c r="R15" s="56" t="n"/>
@@ -15372,6 +15447,7 @@
       <c r="U15" s="56" t="n"/>
       <c r="V15" s="56" t="n"/>
       <c r="W15" s="56" t="n"/>
+      <c r="X15" s="56" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="59" t="inlineStr">
@@ -15424,7 +15500,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O16" s="56" t="n"/>
+      <c r="O16" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P16" s="56" t="n"/>
       <c r="Q16" s="56" t="n"/>
       <c r="R16" s="56" t="n"/>
@@ -15433,6 +15513,7 @@
       <c r="U16" s="56" t="n"/>
       <c r="V16" s="56" t="n"/>
       <c r="W16" s="56" t="n"/>
+      <c r="X16" s="56" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="59" t="inlineStr">
@@ -15489,24 +15570,24 @@
       </c>
       <c r="M17" s="56" t="n"/>
       <c r="N17" s="56" t="n"/>
-      <c r="O17" s="56" t="n"/>
+      <c r="O17" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P17" s="56" t="n"/>
-      <c r="Q17" s="55" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="Q17" s="56" t="n"/>
       <c r="R17" s="55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="S17" s="56" t="n"/>
-      <c r="T17" s="55" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="S17" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T17" s="56" t="n"/>
       <c r="U17" s="55" t="inlineStr">
         <is>
           <t>✓</t>
@@ -15517,7 +15598,12 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W17" s="56" t="n"/>
+      <c r="W17" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X17" s="56" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="59" t="inlineStr">
@@ -15574,24 +15660,24 @@
       </c>
       <c r="M18" s="56" t="n"/>
       <c r="N18" s="56" t="n"/>
-      <c r="O18" s="56" t="n"/>
+      <c r="O18" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P18" s="56" t="n"/>
-      <c r="Q18" s="55" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="Q18" s="56" t="n"/>
       <c r="R18" s="55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="S18" s="56" t="n"/>
-      <c r="T18" s="55" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="S18" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T18" s="56" t="n"/>
       <c r="U18" s="55" t="inlineStr">
         <is>
           <t>✓</t>
@@ -15602,7 +15688,12 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W18" s="56" t="n"/>
+      <c r="W18" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X18" s="56" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="59" t="inlineStr">
@@ -15655,7 +15746,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O19" s="56" t="n"/>
+      <c r="O19" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P19" s="56" t="n"/>
       <c r="Q19" s="56" t="n"/>
       <c r="R19" s="56" t="n"/>
@@ -15664,6 +15759,7 @@
       <c r="U19" s="56" t="n"/>
       <c r="V19" s="56" t="n"/>
       <c r="W19" s="56" t="n"/>
+      <c r="X19" s="56" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="59" t="inlineStr">
@@ -15736,12 +15832,12 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O20" s="56" t="n"/>
-      <c r="P20" s="55" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="O20" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P20" s="56" t="n"/>
       <c r="Q20" s="55" t="inlineStr">
         <is>
           <t>✓</t>
@@ -15773,6 +15869,11 @@
         </is>
       </c>
       <c r="W20" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X20" s="55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -15829,7 +15930,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O21" s="56" t="n"/>
+      <c r="O21" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P21" s="56" t="n"/>
       <c r="Q21" s="56" t="n"/>
       <c r="R21" s="56" t="n"/>
@@ -15838,6 +15943,7 @@
       <c r="U21" s="56" t="n"/>
       <c r="V21" s="56" t="n"/>
       <c r="W21" s="56" t="n"/>
+      <c r="X21" s="56" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="59" t="inlineStr">
@@ -15890,7 +15996,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O22" s="56" t="n"/>
+      <c r="O22" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P22" s="56" t="n"/>
       <c r="Q22" s="56" t="n"/>
       <c r="R22" s="56" t="n"/>
@@ -15899,6 +16009,7 @@
       <c r="U22" s="56" t="n"/>
       <c r="V22" s="56" t="n"/>
       <c r="W22" s="56" t="n"/>
+      <c r="X22" s="56" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="59" t="inlineStr">
@@ -15955,23 +16066,28 @@
       </c>
       <c r="M23" s="56" t="n"/>
       <c r="N23" s="56" t="n"/>
-      <c r="O23" s="56" t="n"/>
+      <c r="O23" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P23" s="56" t="n"/>
       <c r="Q23" s="56" t="n"/>
       <c r="R23" s="56" t="n"/>
-      <c r="S23" s="55" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="S23" s="56" t="n"/>
       <c r="T23" s="55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="U23" s="56" t="n"/>
+      <c r="U23" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="V23" s="56" t="n"/>
-      <c r="W23" s="55" t="inlineStr">
+      <c r="W23" s="56" t="n"/>
+      <c r="X23" s="55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -16032,23 +16148,28 @@
       </c>
       <c r="M24" s="56" t="n"/>
       <c r="N24" s="56" t="n"/>
-      <c r="O24" s="56" t="n"/>
+      <c r="O24" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P24" s="56" t="n"/>
       <c r="Q24" s="56" t="n"/>
       <c r="R24" s="56" t="n"/>
-      <c r="S24" s="55" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="S24" s="56" t="n"/>
       <c r="T24" s="55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="U24" s="56" t="n"/>
+      <c r="U24" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="V24" s="56" t="n"/>
-      <c r="W24" s="55" t="inlineStr">
+      <c r="W24" s="56" t="n"/>
+      <c r="X24" s="55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -16130,12 +16251,12 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P25" s="56" t="n"/>
-      <c r="Q25" s="55" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="P25" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Q25" s="56" t="n"/>
       <c r="R25" s="55" t="inlineStr">
         <is>
           <t>✓</t>
@@ -16162,6 +16283,11 @@
         </is>
       </c>
       <c r="W25" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X25" s="55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -16243,12 +16369,12 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P26" s="56" t="n"/>
-      <c r="Q26" s="55" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="P26" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Q26" s="56" t="n"/>
       <c r="R26" s="55" t="inlineStr">
         <is>
           <t>✓</t>
@@ -16259,18 +16385,23 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="T26" s="56" t="n"/>
-      <c r="U26" s="55" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="T26" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U26" s="56" t="n"/>
       <c r="V26" s="55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
       <c r="W26" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X26" s="55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -16336,7 +16467,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P27" s="56" t="n"/>
+      <c r="P27" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="Q27" s="56" t="n"/>
       <c r="R27" s="56" t="n"/>
       <c r="S27" s="56" t="n"/>
@@ -16344,6 +16479,7 @@
       <c r="U27" s="56" t="n"/>
       <c r="V27" s="56" t="n"/>
       <c r="W27" s="56" t="n"/>
+      <c r="X27" s="56" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="59" t="inlineStr">
@@ -16397,6 +16533,7 @@
       <c r="U28" s="56" t="n"/>
       <c r="V28" s="56" t="n"/>
       <c r="W28" s="56" t="n"/>
+      <c r="X28" s="56" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="59" t="inlineStr">
@@ -16449,7 +16586,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O29" s="56" t="n"/>
+      <c r="O29" s="55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="P29" s="56" t="n"/>
       <c r="Q29" s="56" t="n"/>
       <c r="R29" s="56" t="n"/>
@@ -16458,6 +16599,7 @@
       <c r="U29" s="56" t="n"/>
       <c r="V29" s="56" t="n"/>
       <c r="W29" s="56" t="n"/>
+      <c r="X29" s="56" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="44"/>
@@ -16483,6 +16625,7 @@
       <c r="U30" s="44"/>
       <c r="V30" s="44"/>
       <c r="W30" s="44"/>
+      <c r="X30" s="44"/>
     </row>
     <row r="31">
       <c r="A31" s="45" t="inlineStr">
@@ -16512,6 +16655,7 @@
       <c r="U31" s="44"/>
       <c r="V31" s="44"/>
       <c r="W31" s="44"/>
+      <c r="X31" s="44"/>
     </row>
     <row r="32">
       <c r="A32" s="44"/>
@@ -16537,6 +16681,7 @@
       <c r="U32" s="44"/>
       <c r="V32" s="44"/>
       <c r="W32" s="44"/>
+      <c r="X32" s="44"/>
     </row>
     <row r="33">
       <c r="A33" s="44"/>
@@ -16562,6 +16707,7 @@
       <c r="U33" s="44"/>
       <c r="V33" s="44"/>
       <c r="W33" s="44"/>
+      <c r="X33" s="44"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -16984,7 +17130,7 @@
       </c>
       <c r="B41" t="inlineStr" s="44">
         <is>
-          <t>d2fd7e9</t>
+          <t>023d10e</t>
         </is>
       </c>
     </row>

</xml_diff>